<commit_message>
Adicionado formatação da planilha utilizando Openpyxl deixando a planilha com aparencia mais profissional
</commit_message>
<xml_diff>
--- a/VagasIndeed.xlsx
+++ b/VagasIndeed.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$E$16</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +27,30 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004F81BD"/>
+        <bgColor rgb="004F81BD"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -43,14 +62,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -413,26 +438,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="63" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Título da Vaga</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Data da Coleta</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -441,12 +478,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Estagiário de Dados – Foco em Inteligência Artificial</t>
+          <t>Processo Seletivo 2026 - Cientista de Dados Júnior</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CashMe</t>
+          <t>EloGroup</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -456,19 +493,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=fe524fbea7f5ba1c</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=942f13bf41398652</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Desenvolvedor (a) e Pesquisador (a) de Redes Júnior</t>
+          <t>Processo Seletivo 2026 - Estágio em Ciência de Dados</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Magazine Luiza</t>
+          <t>EloGroup</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -478,19 +520,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=3e6076f3966d44c2</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=f1070129a178a5de</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Desenvolvedor PHP &amp; Python Júnior</t>
+          <t>Processo Seletivo 2026 - Estágio em Engenharia de Dados</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Leega Consultoria</t>
+          <t>EloGroup</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -500,19 +547,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=3fe4ae102798e30b</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=8710c1501a005df4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pessoa desenvolvedora Web Júnior</t>
+          <t>Pessoa Desenvolvedora Backend Python II - Venda Direta</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Terras</t>
+          <t>Grupo Boticário</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -522,19 +574,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=34b10817655112cc</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=e1a13f22b8dca361</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pessoa Desenvolvedora Júnior (Golang, Java, Python)</t>
+          <t>DESENVOLVEDOR PYTHON ESPECIALISTA (Tiviati)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Neogrid Carreiras</t>
+          <t>Jobbol</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -544,19 +601,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=d7826b2cdd2a1c75</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=10b8d9d5d5eff16d</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Python Developer - Ai Training</t>
+          <t>Desenvolvedor (a) e Pesquisador (a) de Redes Júnior</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YO IT CONSULTING</t>
+          <t>Magazine Luiza</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -566,19 +628,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=a30d88b180556284</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=3e6076f3966d44c2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pessoa Desenvolvedora Backend Python II - Venda Direta</t>
+          <t>Desenvolvedor Back-End/APIs Pleno (Java ou Node ou Python)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Grupo Boticário</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -588,19 +655,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=e1a13f22b8dca361</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=a4de1ee83b2715d7</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Python Developer - Analytics and Trading Systems</t>
+          <t>Estagiário - Desenvolvimento</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AlphaCrest Technologies Inc.</t>
+          <t>Nasajon</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -610,19 +682,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=c9b0f3abd6b620cc</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=037409e02bd6bfa1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAS | Analista de Monitoramento de TI JR - Turno Noite</t>
+          <t>Pessoa Desenvolvedora Júnior (Golang, Java, Python)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sicredi</t>
+          <t>Neogrid Carreiras</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -632,19 +709,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=4309bc5155a8efb9</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=d7826b2cdd2a1c75</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Programador JR</t>
+          <t>Desenvolvedor(a) Python com foco em IA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Benner</t>
+          <t>Omie</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -654,19 +736,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=8d30486cf8de7582</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=7fec6bd2c876a33c</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Especialista em IA</t>
+          <t>Desenvolvedor(a) Python</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>COOBRASTUR VIAGENS E TURISMO</t>
+          <t>Omie</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -676,19 +763,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=a47af2eed15c07af</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=bf6ced9602d0a392</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Analytics Engineer Júnior</t>
+          <t>Desenvolvedor Python (foco em dados)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Indicium</t>
+          <t>Safe Consig</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -698,19 +790,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=a26aae1936dc7c65</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=920012dbffbfcfd1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Estagiário - Desenvolvimento</t>
+          <t>Analista de Sistema Pleno (Python) - Remoto</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nasajon</t>
+          <t>Telium Networks</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -720,19 +817,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=037409e02bd6bfa1</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=3204151dccefb66d</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Estágio em QA / Testes de Software</t>
+          <t>Pessoa desenvolvedora Web Júnior</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Radix</t>
+          <t>Terras</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -742,19 +844,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=fef10f74f5fc0a82</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=34b10817655112cc</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Analista de Dados Pleno</t>
+          <t>Python Developer - Ai Training</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Maxxi</t>
+          <t>YO IT CONSULTING</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -764,11 +871,34 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://br.indeed.com/viewjob?jk=733ebe07483ea05f</t>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://br.indeed.com/viewjob?jk=a30d88b180556284</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E16"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>